<commit_message>
Prefer pricing reference info metadata
</commit_message>
<xml_diff>
--- a/templates/pricing-reference/pricing-reference-template.xlsx
+++ b/templates/pricing-reference/pricing-reference-template.xlsx
@@ -3,7 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
     <sheet name="Pricing Reference" sheetId="1" r:id="rId1"/>
-    <sheet name="Instructions" sheetId="2" r:id="rId2"/>
+    <sheet name="Reference Info" sheetId="2" r:id="rId2"/>
+    <sheet name="Instructions" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
@@ -174,7 +175,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B8"/>
   <cols>
     <col min="1" max="1" width="72" customWidth="1"/>
     <col min="2" max="2" width="72" customWidth="1"/>
@@ -183,96 +184,223 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Pricing Reference Import Template</t>
+          <t>Swooshz Pricing Reference Info</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Edit or add pricing rows in the Pricing Reference sheet, then upload this workbook in New Pricing Reference.</t>
+          <t>Reference ID</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t/>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Required columns</t>
+          <t>Reference name</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>section, description, unit_hint, internal_cost, markup_multiplier</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>section</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Quotation section, for example Services.</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>Currency</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Customer-facing wording. Catalog-backed quote basis and output rows will use this exactly.</t>
+          <t>SGD</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>unit_hint</t>
+          <t>Tax label</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Examples: sqm, m length, no, lot, set.</t>
+          <t>GST</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>internal_cost</t>
+          <t>Tax rate</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Number only. This stays internal.</t>
+          <t>0.09</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>markup_multiplier</t>
+          <t>Import note</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Number only, for example 1.5.</t>
+          <t>Edit these values, then upload this workbook through Pricing Reference Settings &gt; Import.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B11"/>
+  <cols>
+    <col min="1" max="1" width="72" customWidth="1"/>
+    <col min="2" max="2" width="72" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Pricing Reference Import Template</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Edit or add pricing rows in the Pricing Reference sheet, then upload this workbook in New Pricing Reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Reference info</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Edit Reference name, Currency, Tax label, and Tax rate in the Reference Info sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Tax rate format</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Use a decimal rate, for example 0.09 for 9% or 0.2 for 20%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Required columns</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>section, description, unit_hint, internal_cost, markup_multiplier</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Quotation section, for example Services.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Customer-facing wording. Catalog-backed quote basis and output rows will use this exactly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>unit_hint</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Examples: sqm, m length, no, lot, set.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>internal_cost</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Number only. This stays internal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>markup_multiplier</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Number only, for example 1.5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>remarks</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Optional. Internal matching/search notes; separate multiple values with semicolon. AI-generated aliases are added during import.</t>
         </is>

</xml_diff>

<commit_message>
Refresh output downloads after row edits
</commit_message>
<xml_diff>
--- a/templates/pricing-reference/pricing-reference-template.xlsx
+++ b/templates/pricing-reference/pricing-reference-template.xlsx
@@ -11,14 +11,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:H4"/>
   <cols>
     <col min="1" max="1" width="0" hidden="1" customWidth="1"/>
-    <col min="2" max="2" width="24" customWidth="1"/>
-    <col min="3" max="3" width="72" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="6" width="18" customWidth="1"/>
-    <col min="7" max="7" width="36" customWidth="1"/>
+    <col min="2" max="2" width="10" customWidth="1"/>
+    <col min="3" max="3" width="24" customWidth="1"/>
+    <col min="4" max="4" width="72" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="7" width="18" customWidth="1"/>
+    <col min="8" max="8" width="36" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -29,30 +30,35 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>row</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>section</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>unit_hint</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>internal_cost</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>markup_multiplier</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>remarks</t>
         </is>
@@ -66,30 +72,35 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>Services</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>lot standard project coordination</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>lot</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>1.2</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>example service row</t>
         </is>
@@ -103,30 +114,35 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>Materials</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>sqm standard surface finish</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>sqm</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>1.5</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>example area-based material row</t>
         </is>
@@ -140,30 +156,35 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>Equipment Rental</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>nos. standard device rental</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>nos</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>50</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>1.5</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>example rental row</t>
         </is>
@@ -278,7 +299,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <cols>
     <col min="1" max="1" width="72" customWidth="1"/>
     <col min="2" max="2" width="72" customWidth="1"/>
@@ -337,70 +358,82 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>section</t>
+          <t>row</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Quotation section, for example Services.</t>
+          <t>Optional display/order number. Rows with lower numbers appear earlier in the imported reference.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>section</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Customer-facing wording. Catalog-backed quote basis and output rows will use this exactly.</t>
+          <t>Quotation section, for example Services.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>unit_hint</t>
+          <t>description</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Examples: sqm, m length, no, lot, set.</t>
+          <t>Customer-facing wording. Catalog-backed quote basis and output rows will use this exactly.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>internal_cost</t>
+          <t>unit_hint</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Number only. This stays internal.</t>
+          <t>Examples: sqm, m length, no, lot, set.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>markup_multiplier</t>
+          <t>internal_cost</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Number only, for example 1.5.</t>
+          <t>Number only. This stays internal.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>markup_multiplier</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Number only, for example 1.5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>remarks</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>Optional. Internal matching/search notes; separate multiple values with semicolon. AI-generated aliases are added during import.</t>
         </is>

</xml_diff>